<commit_message>
feat: operateurs/villes lookup, devis polish, responsive fixes
- devis-api: add /api/operateurs and /api/villes endpoints, drop the
  old unused api/ module in favor of devis-api
- devis_template.xlsx: fix "Tarifs de référence" text clipping and
  "Total de la commande" spacing, auto-fill "NANTERRE Le" with the
  order date
- frontend: generated PDF opens in a new window instead of forcing a
  download; "Ouvrir Outlook" opens a prefilled mailto: email
  independently from PDF generation; replace hardcoded arrow with an
  SVG icon; make the prestations list responsive on mobile
</commit_message>
<xml_diff>
--- a/devis-api/template/devis_template.xlsx
+++ b/devis-api/template/devis_template.xlsx
@@ -1609,7 +1609,7 @@
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+      <alignment horizontal="right" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -1648,7 +1648,7 @@
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>

</xml_diff>